<commit_message>
docs: correct confirmed human review process and record intake findings
Record the project owner's 2026-10-20 confirmation of two independent human final reviews. Change process declarations only, preserve judgments and original history, refresh exact-byte hashes, and document remaining structural issues and development-only agreement.
</commit_message>
<xml_diff>
--- a/监管RAG第一阶段双人复核_20261019/submissions/reviewer_A-7402/real10/复核表.xlsx
+++ b/监管RAG第一阶段双人复核_20261019/submissions/reviewer_A-7402/real10/复核表.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M2" s="11" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M3" s="11" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M4" s="11" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M5" s="11" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M6" s="11" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M7" s="11" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M9" s="11" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M10" s="11" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>独立填写；提交前未查看另一复核人表格或判断；未使用包外材料</t>
+          <t>本人逐条核对原文后确认本表；提交前未查看另一复核人员判断。过程声明依据项目负责人2026-10-20确认更正。</t>
         </is>
       </c>
       <c r="M11" s="11" t="inlineStr">

</xml_diff>